<commit_message>
feat: adiciona código para PL Tabata Amaral
</commit_message>
<xml_diff>
--- a/tables/resultados_distributivos_com_arrecadacao.xlsx
+++ b/tables/resultados_distributivos_com_arrecadacao.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -489,6 +489,31 @@
       </c>
       <c r="G5">
         <v>78.88719703757363</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Proposta - Tabata</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>0.6117819059067546</v>
+      </c>
+      <c r="C6">
+        <v>0.1424354334895495</v>
+      </c>
+      <c r="D6">
+        <v>0.5410060227090372</v>
+      </c>
+      <c r="E6">
+        <v>0.2326304856684225</v>
+      </c>
+      <c r="F6">
+        <v>441.5333436408516</v>
+      </c>
+      <c r="G6">
+        <v>106.8377657556875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>